<commit_message>
build(currency-wars): G12-P3-B6 verify Sora workbook pipeline
</commit_message>
<xml_diff>
--- a/config/currency-wars-generated/templates/CurrencyWarsReview.xlsx
+++ b/config/currency-wars-generated/templates/CurrencyWarsReview.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="91">
   <si>
     <t>@table</t>
   </si>
@@ -52,7 +52,7 @@
     <t>@schema</t>
   </si>
   <si>
-    <t>c62b826feea99301</t>
+    <t>daf1db96530d9b59</t>
   </si>
   <si>
     <t>#name</t>
@@ -118,6 +118,9 @@
     <t>string</t>
   </si>
   <si>
+    <t>optional&lt;string&gt;</t>
+  </si>
+  <si>
     <t>#scope</t>
   </si>
   <si>
@@ -130,19 +133,13 @@
     <t>length=1..32767</t>
   </si>
   <si>
-    <t>length=2..32767</t>
-  </si>
-  <si>
-    <t>length=0..32767</t>
-  </si>
-  <si>
     <t>#desc</t>
   </si>
   <si>
     <t>CurrencyWarsMechanicRules</t>
   </si>
   <si>
-    <t>48025e0283ae12d6</t>
+    <t>6f3f7703879e67b3</t>
   </si>
   <si>
     <t>scope</t>
@@ -163,7 +160,7 @@
     <t>CurrencyWarsSources</t>
   </si>
   <si>
-    <t>104b4387cfb5475d</t>
+    <t>cce8fc2ef8695d9f</t>
   </si>
   <si>
     <t>repository</t>
@@ -187,7 +184,7 @@
     <t>CurrencyWarsCoverage</t>
   </si>
   <si>
-    <t>fa177f60e2552b67</t>
+    <t>c7866196933a4545</t>
   </si>
   <si>
     <t>manifest_category</t>
@@ -205,7 +202,7 @@
     <t>CurrencyWarsResearchGaps</t>
   </si>
   <si>
-    <t>f700b6c0ec23f315</t>
+    <t>0bbdaf2749fa8726</t>
   </si>
   <si>
     <t>field</t>
@@ -226,7 +223,7 @@
     <t>CurrencyWarsSemanticFixtureFamilies</t>
   </si>
   <si>
-    <t>aa8a175b53f6af8b</t>
+    <t>61d9eb73022a9cc5</t>
   </si>
   <si>
     <t>minimum_cases</t>
@@ -238,7 +235,7 @@
     <t>CurrencyWarsReviewFixtures</t>
   </si>
   <si>
-    <t>6a8cb8e2de8344e5</t>
+    <t>5f636a2eb2b65532</t>
   </si>
   <si>
     <t>family_id</t>
@@ -256,7 +253,7 @@
     <t>CurrencyWarsReconciliationReceipts</t>
   </si>
   <si>
-    <t>8bfea203a32125bb</t>
+    <t>d113a1fc61d556b4</t>
   </si>
   <si>
     <t>row_locator</t>
@@ -274,7 +271,7 @@
     <t>CurrencyWarsManifest</t>
   </si>
   <si>
-    <t>ad642d5c59a54c57</t>
+    <t>d6e8a7e333c8a630</t>
   </si>
   <si>
     <t>content_manifest_sha256</t>
@@ -289,7 +286,7 @@
     <t>CurrencyWarsPackIndex</t>
   </si>
   <si>
-    <t>dc5b7058678b1f29</t>
+    <t>c721f7024c1c700e</t>
   </si>
   <si>
     <t>pack_digest</t>
@@ -726,10 +723,8 @@
     <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="15" width="12.7109375" style="5" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="15.7109375" style="5" customWidth="1"/>
-    <col min="18" max="18" width="12.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="18" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -920,21 +915,21 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:18">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -990,40 +985,40 @@
     </row>
     <row r="6" spans="1:18">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -1032,21 +1027,21 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1090,8 +1085,8 @@
     <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="16" width="12.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="15.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="17" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -1099,7 +1094,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1123,7 +1118,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -1170,13 +1165,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -1223,13 +1218,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>90</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -1276,18 +1271,18 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -1340,40 +1335,40 @@
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -1382,18 +1377,18 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1436,9 +1431,10 @@
     <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="16" width="12.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="16" width="16.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="18.7109375" style="5" customWidth="1"/>
-    <col min="18" max="19" width="15.7109375" style="5" customWidth="1"/>
+    <col min="18" max="19" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -1446,7 +1442,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1470,7 +1466,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -1517,19 +1513,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -1576,19 +1572,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="R3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="S3" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -1635,24 +1631,24 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -1711,40 +1707,40 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -1753,24 +1749,24 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -1815,7 +1811,8 @@
     <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="19" width="12.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="19" width="16.7109375" style="5" customWidth="1"/>
     <col min="20" max="20" width="17.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1824,7 +1821,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -1848,7 +1845,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="24" customHeight="1">
@@ -1895,22 +1892,22 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="S2" s="3" t="s">
+      <c r="T2" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:20">
@@ -1957,22 +1954,22 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="R3" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="S3" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="T3" s="5" t="s">
         <v>51</v>
-      </c>
-      <c r="T3" s="5" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:20">
@@ -2019,27 +2016,27 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:20">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -2101,40 +2098,40 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -2143,27 +2140,27 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2213,7 +2210,7 @@
     <col min="15" max="15" width="17.7109375" style="5" customWidth="1"/>
     <col min="16" max="16" width="18.7109375" style="5" customWidth="1"/>
     <col min="17" max="17" width="21.7109375" style="5" customWidth="1"/>
-    <col min="18" max="18" width="12.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18">
@@ -2221,7 +2218,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2245,7 +2242,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="24" customHeight="1">
@@ -2292,16 +2289,16 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:18">
@@ -2348,16 +2345,16 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="R3" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:18">
@@ -2404,21 +2401,21 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:18">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -2474,40 +2471,40 @@
     </row>
     <row r="6" spans="1:18">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -2516,21 +2513,21 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2574,9 +2571,8 @@
     <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="16" width="12.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="15.7109375" style="5" customWidth="1"/>
-    <col min="18" max="18" width="12.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="18" width="16.7109375" style="5" customWidth="1"/>
     <col min="19" max="19" width="21.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2585,7 +2581,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2609,7 +2605,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -2656,19 +2652,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -2715,19 +2711,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="R3" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="S3" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -2774,24 +2770,24 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -2850,40 +2846,40 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -2892,24 +2888,24 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -2955,8 +2951,7 @@
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" style="5" customWidth="1"/>
-    <col min="16" max="16" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="16" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -2964,7 +2959,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2988,7 +2983,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="24" customHeight="1">
@@ -3035,10 +3030,10 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -3085,10 +3080,10 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="P3" s="5" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -3135,15 +3130,15 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -3193,40 +3188,40 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -3235,15 +3230,15 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -3285,11 +3280,10 @@
     <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="15" width="12.7109375" style="5" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="12.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="17" width="16.7109375" style="5" customWidth="1"/>
     <col min="18" max="18" width="18.7109375" style="5" customWidth="1"/>
-    <col min="19" max="19" width="14.7109375" style="5" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -3297,7 +3291,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3321,7 +3315,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -3368,19 +3362,19 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -3427,19 +3421,19 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="R3" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="S3" s="5" t="s">
         <v>74</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -3486,24 +3480,24 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -3562,40 +3556,40 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -3604,24 +3598,24 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -3666,9 +3660,8 @@
     <col min="10" max="10" width="12.7109375" style="5" customWidth="1"/>
     <col min="11" max="11" width="14.7109375" style="5" customWidth="1"/>
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
-    <col min="14" max="16" width="12.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="15.7109375" style="5" customWidth="1"/>
-    <col min="18" max="19" width="12.7109375" style="5" customWidth="1"/>
+    <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
+    <col min="15" max="19" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
@@ -3676,7 +3669,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3700,7 +3693,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="24" customHeight="1">
@@ -3750,16 +3743,16 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q2" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="Q2" s="3" t="s">
+      <c r="R2" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="R2" s="3" t="s">
+      <c r="S2" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="S2" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -3809,16 +3802,16 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="Q3" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="R3" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="S3" s="5" t="s">
         <v>80</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:19">
@@ -3865,24 +3858,24 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:19">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -3941,40 +3934,40 @@
     </row>
     <row r="6" spans="1:19">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -3983,24 +3976,24 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:19" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -4047,8 +4040,7 @@
     <col min="12" max="13" width="16.7109375" style="5" customWidth="1"/>
     <col min="14" max="14" width="12.7109375" style="5" customWidth="1"/>
     <col min="15" max="15" width="23.7109375" style="5" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" style="5" customWidth="1"/>
-    <col min="17" max="17" width="13.7109375" style="5" customWidth="1"/>
+    <col min="16" max="17" width="16.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
@@ -4056,7 +4048,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4080,7 +4072,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="24" customHeight="1">
@@ -4127,13 +4119,13 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="P2" s="3" t="s">
+      <c r="Q2" s="3" t="s">
         <v>85</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:17">
@@ -4180,13 +4172,13 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="P3" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>85</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:17">
@@ -4233,18 +4225,18 @@
         <v>30</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="A5" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>7</v>
@@ -4297,40 +4289,40 @@
     </row>
     <row r="6" spans="1:17">
       <c r="A6" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M6" s="5" t="s">
         <v>35</v>
@@ -4339,18 +4331,18 @@
         <v>35</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>

</xml_diff>